<commit_message>
n1 small refactor and updated keycodes.xlsx
</commit_message>
<xml_diff>
--- a/docs/keycodes.xlsx
+++ b/docs/keycodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://siemens-my.sharepoint.com/personal/michael_loos_siemens_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\homod\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D659703-BFB8-4E3E-BBF0-46AC800B59BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E923E5F-28FD-469B-BAB1-CE29AFD251BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8E0E9403-79CF-4D40-9769-565AD34A791E}"/>
+    <workbookView xWindow="8670" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{8E0E9403-79CF-4D40-9769-565AD34A791E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>+</t>
   </si>
@@ -219,16 +219,56 @@
   </si>
   <si>
     <t>&amp;kp TILDE2</t>
+  </si>
+  <si>
+    <t>LS(NON_US_BACKSLASH)</t>
+  </si>
+  <si>
+    <t>output</t>
+  </si>
+  <si>
+    <t>Keycode</t>
+  </si>
+  <si>
+    <t>LS(NON_US_HASH)</t>
+  </si>
+  <si>
+    <t>´</t>
+  </si>
+  <si>
+    <t>~</t>
+  </si>
+  <si>
+    <t>&amp;kp LESS_THAN</t>
+  </si>
+  <si>
+    <t>&amp;kp RA(RBKT)</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>&amp;kp PLUS</t>
+  </si>
+  <si>
+    <t>&amp;kp RA(NON_US_BACKSLASH)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -254,9 +294,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -591,252 +632,312 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD80ACD5-7E64-4F5B-B82F-4B333B2F6D30}">
-  <dimension ref="A1:Q27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.21875" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>37</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="s">
         <v>48</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>38</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" t="s">
         <v>43</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>39</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>44</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>40</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E5" t="s">
         <v>45</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>59</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
         <v>46</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>22</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E7" t="s">
         <v>47</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" t="s">
         <v>54</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>32</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C21" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>55</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>56</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="Q27" s="1"/>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>